<commit_message>
fabrication checkboxes + stock alerts + dedup import
</commit_message>
<xml_diff>
--- a/LISTE DES PRODUITS FINI.xlsx
+++ b/LISTE DES PRODUITS FINI.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10308"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D66B7672-99EE-1B45-ABAB-B82731071C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="22260" windowHeight="12640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LISTE PRODUIT FINI AU 30062026" sheetId="3" r:id="rId1"/>
@@ -12,17 +13,28 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LISTE PRODUIT FINI AU 30062026'!$B$5:$E$122</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="173">
   <si>
     <t>CONCEPTION RIDELLE</t>
   </si>
@@ -535,14 +547,20 @@
   </si>
   <si>
     <t>DPR00203</t>
+  </si>
+  <si>
+    <t>DPR0006</t>
+  </si>
+  <si>
+    <t>DPR0029</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -594,18 +612,18 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Milliers" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -883,17 +901,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:E89"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="63" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.5" customWidth="1"/>
+    <col min="5" max="5" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B2" s="3" t="s">
         <v>88</v>
       </c>
@@ -901,7 +919,7 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>17</v>
       </c>
@@ -915,7 +933,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>89</v>
       </c>
@@ -933,7 +951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>90</v>
       </c>
@@ -951,7 +969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>92</v>
       </c>
@@ -969,7 +987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>94</v>
       </c>
@@ -987,7 +1005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>95</v>
       </c>
@@ -1005,9 +1023,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>171</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>25</v>
@@ -1023,7 +1041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>91</v>
       </c>
@@ -1041,7 +1059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>93</v>
       </c>
@@ -1059,7 +1077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1077,7 +1095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>97</v>
       </c>
@@ -1095,7 +1113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>167</v>
       </c>
@@ -1113,7 +1131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>98</v>
       </c>
@@ -1131,7 +1149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>106</v>
       </c>
@@ -1149,7 +1167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>99</v>
       </c>
@@ -1167,7 +1185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>166</v>
       </c>
@@ -1185,7 +1203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>100</v>
       </c>
@@ -1203,7 +1221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>101</v>
       </c>
@@ -1221,7 +1239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>164</v>
       </c>
@@ -1239,7 +1257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>102</v>
       </c>
@@ -1257,7 +1275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>103</v>
       </c>
@@ -1275,7 +1293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>104</v>
       </c>
@@ -1293,7 +1311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>165</v>
       </c>
@@ -1311,7 +1329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>168</v>
       </c>
@@ -1329,7 +1347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>105</v>
       </c>
@@ -1347,7 +1365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>169</v>
       </c>
@@ -1365,7 +1383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>107</v>
       </c>
@@ -1383,7 +1401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -1401,7 +1419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>109</v>
       </c>
@@ -1419,9 +1437,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>172</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>11</v>
@@ -1437,7 +1455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>110</v>
       </c>
@@ -1455,7 +1473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>111</v>
       </c>
@@ -1473,7 +1491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>112</v>
       </c>
@@ -1491,7 +1509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>113</v>
       </c>
@@ -1509,7 +1527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>114</v>
       </c>
@@ -1527,7 +1545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>115</v>
       </c>
@@ -1545,7 +1563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>116</v>
       </c>
@@ -1563,7 +1581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>117</v>
       </c>
@@ -1581,7 +1599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>118</v>
       </c>
@@ -1599,7 +1617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>119</v>
       </c>
@@ -1617,7 +1635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>120</v>
       </c>
@@ -1635,7 +1653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>121</v>
       </c>
@@ -1653,7 +1671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>122</v>
       </c>
@@ -1671,7 +1689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>123</v>
       </c>
@@ -1689,7 +1707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>124</v>
       </c>
@@ -1707,7 +1725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>125</v>
       </c>
@@ -1725,7 +1743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>126</v>
       </c>
@@ -1743,7 +1761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>127</v>
       </c>
@@ -1761,7 +1779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>128</v>
       </c>
@@ -1779,7 +1797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>129</v>
       </c>
@@ -1797,7 +1815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>130</v>
       </c>
@@ -1815,7 +1833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>131</v>
       </c>
@@ -1833,7 +1851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>132</v>
       </c>
@@ -1851,7 +1869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>133</v>
       </c>
@@ -1869,7 +1887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>134</v>
       </c>
@@ -1887,7 +1905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>135</v>
       </c>
@@ -1905,7 +1923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>136</v>
       </c>
@@ -1923,7 +1941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>137</v>
       </c>
@@ -1941,7 +1959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>138</v>
       </c>
@@ -1959,7 +1977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>139</v>
       </c>
@@ -1977,7 +1995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>140</v>
       </c>
@@ -1995,7 +2013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>141</v>
       </c>
@@ -2013,7 +2031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>142</v>
       </c>
@@ -2031,7 +2049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>143</v>
       </c>
@@ -2049,7 +2067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>144</v>
       </c>
@@ -2067,7 +2085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>145</v>
       </c>
@@ -2085,7 +2103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>146</v>
       </c>
@@ -2103,7 +2121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>147</v>
       </c>
@@ -2121,7 +2139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>148</v>
       </c>
@@ -2139,7 +2157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>149</v>
       </c>
@@ -2157,7 +2175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>150</v>
       </c>
@@ -2175,7 +2193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>151</v>
       </c>
@@ -2193,7 +2211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>152</v>
       </c>
@@ -2211,7 +2229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>153</v>
       </c>
@@ -2229,7 +2247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>154</v>
       </c>
@@ -2247,7 +2265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>155</v>
       </c>
@@ -2265,7 +2283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>156</v>
       </c>
@@ -2283,7 +2301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>157</v>
       </c>
@@ -2301,7 +2319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>158</v>
       </c>
@@ -2319,7 +2337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>159</v>
       </c>
@@ -2337,7 +2355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>160</v>
       </c>
@@ -2355,7 +2373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>161</v>
       </c>
@@ -2373,7 +2391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>170</v>
       </c>
@@ -2391,7 +2409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>162</v>
       </c>
@@ -2409,7 +2427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>163</v>
       </c>
@@ -2427,7 +2445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E89" s="2"/>
     </row>
   </sheetData>

</xml_diff>